<commit_message>
#4 Both Transmitter and Receiver PCB Completed with Deliverables
</commit_message>
<xml_diff>
--- a/Design-Files/TYPE-C_4K_TRANSMITTER-v1.0/BOM/Client BOM - TYPEC_4KTransmitter-v1.0.xlsx
+++ b/Design-Files/TYPE-C_4K_TRANSMITTER-v1.0/BOM/Client BOM - TYPEC_4KTransmitter-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\aaronsushinsky-wirelesshdmi-hw\Design-Files\TYPE-C_4K_TRANSMITTER-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34CB1E73-B470-4A79-AE9C-900A6F676D1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E133561-A7BD-46EA-90B2-9A895A792F08}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="449">
   <si>
     <t>#</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>[NoParam], Capacitor</t>
-  </si>
-  <si>
     <t>Diode</t>
   </si>
   <si>
@@ -226,7 +223,7 @@
     <t>R1, R43</t>
   </si>
   <si>
-    <t>R2, R51, R95, R124</t>
+    <t>R2, R28, R51, R95, R124</t>
   </si>
   <si>
     <t>R3, R29, R45, R50, R56, R87, R93, R114, R115, R116, R117, R140, R169, R170, R171, R172, R173, R174, R175, R176</t>
@@ -526,7 +523,7 @@
     <t>RES 1M OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 22 OHM 1% 1/16W 0402, RES 10K OHM 1% 1/16W 0402, RES 4.7K OHM 1% 1/16W 0402</t>
+    <t>RES 22 OHM 1% 1/16W 0402, RES 0 OHM JUMPER 1/16W 0402, RES 10K OHM 1% 1/16W 0402, RES 4.7K OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 0 OHM JUMPER 1/16W 0402</t>
@@ -637,7 +634,7 @@
     <t>IC INTERFACE SPECIALIZED 24UQFN</t>
   </si>
   <si>
-    <t>FBGA-153(11.5x13) eMMC ROHS</t>
+    <t>eMMC 5.1 FBGA-153 eMMC ROHS</t>
   </si>
   <si>
     <t>5.4Gbps Type-C/DP/eDPToDual-port MIPI DSI/CSI/LVDS with Audio QFN-64(7.5x7.5) Video Interface ICs ROHS</t>
@@ -793,7 +790,7 @@
     <t>SOT-23-5</t>
   </si>
   <si>
-    <t>200-WFBGA (10x14.5)</t>
+    <t>200-WFBGA (10x15)</t>
   </si>
   <si>
     <t>AP6275S_</t>
@@ -931,7 +928,7 @@
     <t>RC0402FR-071ML</t>
   </si>
   <si>
-    <t>RC0402FR-0722RL, RC0402FR-0710KL, RC0402FR-074K7L</t>
+    <t>RC0402FR-0722RL, RC0402FR-070RL, RC0402FR-0710KL, RC0402FR-074K7L</t>
   </si>
   <si>
     <t>RC0402FR-070RL</t>
@@ -1042,7 +1039,7 @@
     <t>TPD12S016RKTR</t>
   </si>
   <si>
-    <t>KLM8G1GETF-B041</t>
+    <t>KLMAG1JETD-B041</t>
   </si>
   <si>
     <t>LT7911D</t>
@@ -1063,7 +1060,7 @@
     <t>SY8089AAAC</t>
   </si>
   <si>
-    <t>K4UBE3D4AA-MGCL</t>
+    <t>K4U6E3S4AA-MGCL</t>
   </si>
   <si>
     <t>TLV62569DBVR</t>
@@ -1897,25 +1894,25 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1928,22 +1925,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1959,22 +1956,22 @@
         <v>3</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="J4" s="9">
         <v>9</v>
@@ -1990,22 +1987,22 @@
         <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J5" s="7">
         <v>57</v>
@@ -2018,25 +2015,25 @@
         <v>4</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="J6" s="9">
         <v>17</v>
@@ -2052,22 +2049,22 @@
         <v>3</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -2083,22 +2080,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J8" s="9">
         <v>2</v>
@@ -2114,22 +2111,22 @@
         <v>3</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -2142,25 +2139,25 @@
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J10" s="9">
         <v>22</v>
@@ -2176,22 +2173,22 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -2207,22 +2204,22 @@
         <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J12" s="9">
         <v>25</v>
@@ -2238,22 +2235,22 @@
         <v>3</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J13" s="7">
         <v>31</v>
@@ -2269,22 +2266,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="J14" s="9">
         <v>18</v>
@@ -2300,22 +2297,22 @@
         <v>3</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
@@ -2331,22 +2328,22 @@
         <v>3</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J16" s="9">
         <v>3</v>
@@ -2362,22 +2359,22 @@
         <v>3</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2393,22 +2390,22 @@
         <v>3</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2424,22 +2421,22 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J19" s="7">
         <v>64</v>
@@ -2455,22 +2452,22 @@
         <v>3</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="J20" s="9">
         <v>7</v>
@@ -2486,22 +2483,22 @@
         <v>3</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J21" s="7">
         <v>2</v>
@@ -2517,22 +2514,22 @@
         <v>3</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="J22" s="9">
         <v>4</v>
@@ -2548,22 +2545,22 @@
         <v>3</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J23" s="7">
         <v>4</v>
@@ -2579,22 +2576,22 @@
         <v>3</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -2610,22 +2607,22 @@
         <v>3</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2641,22 +2638,22 @@
         <v>3</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2669,25 +2666,25 @@
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J27" s="7">
         <v>8</v>
@@ -2700,25 +2697,25 @@
         <v>26</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J28" s="9">
         <v>2</v>
@@ -2731,25 +2728,25 @@
         <v>27</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J29" s="7">
         <v>2</v>
@@ -2762,25 +2759,25 @@
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2793,25 +2790,25 @@
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J31" s="7">
         <v>6</v>
@@ -2824,25 +2821,25 @@
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2855,25 +2852,25 @@
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J33" s="7">
         <v>2</v>
@@ -2886,25 +2883,25 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2917,25 +2914,25 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2948,25 +2945,25 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J36" s="9">
         <v>2</v>
@@ -2979,25 +2976,25 @@
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -3010,25 +3007,25 @@
         <v>36</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="J38" s="9">
         <v>5</v>
@@ -3041,25 +3038,25 @@
         <v>37</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F39" s="7">
         <v>302</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J39" s="7">
         <v>2</v>
@@ -3072,25 +3069,25 @@
         <v>38</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -3103,25 +3100,25 @@
         <v>39</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -3134,25 +3131,25 @@
         <v>40</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -3165,25 +3162,25 @@
         <v>41</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
@@ -3196,25 +3193,25 @@
         <v>42</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -3227,25 +3224,25 @@
         <v>43</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
@@ -3258,59 +3255,59 @@
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="J46" s="9">
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
         <v>45</v>
       </c>
-      <c r="C47" s="12" t="s">
-        <v>15</v>
+      <c r="C47" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J47" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3319,26 +3316,26 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C48" s="12" t="s">
-        <v>15</v>
+      <c r="C48" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J48" s="9">
         <v>20</v>
@@ -3351,25 +3348,25 @@
         <v>47</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="J49" s="7">
         <v>2</v>
@@ -3382,25 +3379,25 @@
         <v>48</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J50" s="9">
         <v>5</v>
@@ -3412,26 +3409,26 @@
         <f>ROW(B51) - ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="12" t="s">
-        <v>15</v>
+      <c r="C51" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="J51" s="7">
         <v>2</v>
@@ -3444,25 +3441,25 @@
         <v>50</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3475,25 +3472,25 @@
         <v>51</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="J53" s="7">
         <v>8</v>
@@ -3506,25 +3503,25 @@
         <v>52</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3537,25 +3534,25 @@
         <v>53</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J55" s="7">
         <v>1</v>
@@ -3568,25 +3565,25 @@
         <v>54</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3599,25 +3596,25 @@
         <v>55</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="J57" s="7">
         <v>7</v>
@@ -3630,25 +3627,25 @@
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J58" s="9">
         <v>2</v>
@@ -3661,25 +3658,25 @@
         <v>57</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3692,25 +3689,25 @@
         <v>58</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="J60" s="9">
         <v>9</v>
@@ -3723,25 +3720,25 @@
         <v>59</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="J61" s="7">
         <v>7</v>
@@ -3754,25 +3751,25 @@
         <v>60</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="J62" s="9">
         <v>1</v>
@@ -3785,25 +3782,25 @@
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3816,25 +3813,25 @@
         <v>62</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J64" s="9">
         <v>1</v>
@@ -3847,25 +3844,25 @@
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="J65" s="7">
         <v>2</v>
@@ -3878,25 +3875,25 @@
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3908,26 +3905,24 @@
         <f>ROW(B67) - ROW($B$2)</f>
         <v>65</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="C67" s="12"/>
       <c r="D67" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J67" s="7">
         <v>5</v>
@@ -3940,25 +3935,25 @@
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="J68" s="9">
         <v>1</v>
@@ -3971,25 +3966,25 @@
         <v>67</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J69" s="7">
         <v>3</v>
@@ -4002,25 +3997,25 @@
         <v>68</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="J70" s="9">
         <v>1</v>
@@ -4032,26 +4027,26 @@
         <f>ROW(B71) - ROW($B$2)</f>
         <v>69</v>
       </c>
-      <c r="C71" s="12" t="s">
-        <v>15</v>
+      <c r="C71" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="J71" s="7">
         <v>2</v>
@@ -4063,26 +4058,26 @@
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="C72" s="12" t="s">
-        <v>15</v>
+      <c r="C72" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="J72" s="9">
         <v>5</v>
@@ -4095,25 +4090,25 @@
         <v>71</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="J73" s="7">
         <v>8</v>
@@ -4126,25 +4121,25 @@
         <v>72</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4157,25 +4152,25 @@
         <v>73</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J75" s="7">
         <v>2</v>
@@ -4188,25 +4183,25 @@
         <v>74</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4219,25 +4214,25 @@
         <v>75</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="J77" s="7">
         <v>1</v>
@@ -4249,26 +4244,26 @@
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="C78" s="12" t="s">
-        <v>15</v>
+      <c r="C78" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="J78" s="9">
         <v>2</v>
@@ -4281,25 +4276,25 @@
         <v>77</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4312,25 +4307,25 @@
         <v>78</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F80" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G80" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I80" s="10" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="J80" s="9">
         <v>2</v>
@@ -4343,25 +4338,25 @@
         <v>79</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="J81" s="7">
         <v>2</v>
@@ -4373,26 +4368,24 @@
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="C82" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="C82" s="13"/>
       <c r="D82" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I82" s="10" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="J82" s="9">
         <v>5</v>
@@ -4405,25 +4398,25 @@
         <v>81</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J83" s="7">
         <v>3</v>
@@ -4436,25 +4429,25 @@
         <v>82</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F84" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H84" s="9" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="I84" s="10" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J84" s="9">
         <v>1</v>
@@ -4467,25 +4460,25 @@
         <v>83</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H85" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J85" s="7">
         <v>1</v>
@@ -4499,22 +4492,22 @@
       </c>
       <c r="C86" s="13"/>
       <c r="D86" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H86" s="9" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I86" s="10" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J86" s="9">
         <v>1</v>
@@ -4527,25 +4520,25 @@
         <v>85</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H87" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I87" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J87" s="7">
         <v>1</v>
@@ -4558,25 +4551,25 @@
         <v>86</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F88" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H88" s="9" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="I88" s="10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J88" s="9">
         <v>1</v>
@@ -4589,25 +4582,25 @@
         <v>87</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H89" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J89" s="7">
         <v>1</v>
@@ -4620,25 +4613,25 @@
         <v>88</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F90" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G90" s="10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H90" s="9" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I90" s="10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J90" s="9">
         <v>1</v>
@@ -4651,25 +4644,25 @@
         <v>89</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H91" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I91" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J91" s="7">
         <v>1</v>
@@ -4682,25 +4675,25 @@
         <v>90</v>
       </c>
       <c r="C92" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D92" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F92" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G92" s="10" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H92" s="9" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="I92" s="10" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="J92" s="9">
         <v>1</v>
@@ -4713,25 +4706,25 @@
         <v>91</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D93" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G93" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="H93" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="I93" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J93" s="7">
         <v>1</v>
@@ -4744,25 +4737,25 @@
         <v>92</v>
       </c>
       <c r="C94" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F94" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G94" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H94" s="9" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I94" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J94" s="9">
         <v>1</v>
@@ -4775,25 +4768,25 @@
         <v>93</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G95" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H95" s="7" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I95" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J95" s="7">
         <v>1</v>
@@ -4806,25 +4799,25 @@
         <v>94</v>
       </c>
       <c r="C96" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F96" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G96" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H96" s="9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I96" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J96" s="9">
         <v>1</v>
@@ -4837,25 +4830,25 @@
         <v>95</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G97" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H97" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="I97" s="8" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="J97" s="7">
         <v>1</v>
@@ -4868,25 +4861,25 @@
         <v>96</v>
       </c>
       <c r="C98" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D98" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F98" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G98" s="10" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H98" s="9" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I98" s="10" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="J98" s="9">
         <v>1</v>
@@ -4899,25 +4892,25 @@
         <v>97</v>
       </c>
       <c r="C99" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F99" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G99" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H99" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="I99" s="8" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="J99" s="7">
         <v>1</v>
@@ -4930,25 +4923,25 @@
         <v>98</v>
       </c>
       <c r="C100" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D100" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E100" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F100" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="G100" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H100" s="9" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="I100" s="10" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="J100" s="9">
         <v>1</v>
@@ -4961,25 +4954,25 @@
         <v>99</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="I101" s="8" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="J101" s="7">
         <v>1</v>

</xml_diff>